<commit_message>
Add combined 自アポ+IS 有効提案取得 count and rate to 課長報告
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2eWcGBYWFrU2WgTZUGmvP
</commit_message>
<xml_diff>
--- a/jiho/時報シート_SL東京1部1課.xlsx
+++ b/jiho/時報シート_SL東京1部1課.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="41">
   <si>
     <t xml:space="preserve">時報入力シート</t>
   </si>
@@ -372,6 +372,36 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得（自アポ＋</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IS</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合算）</t>
     </r>
   </si>
   <si>
@@ -1989,13 +2019,15 @@
         <v>23</v>
       </c>
       <c r="F5" s="15" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"12時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B6&amp;" / "&amp;C6&amp;" = "&amp;IF(N(C6)=0,"-",TEXT(B6/C6,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B7&amp;" / "&amp;C7&amp;" = "&amp;IF(N(C7)=0,"-",TEXT(B7/C7,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B8&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B9&amp;"件"</f>
+        <f aca="false">"【"&amp;設定!$B$4&amp;"12時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B6&amp;" / "&amp;C6&amp;" = "&amp;IF(N(C6)=0,"-",TEXT(B6/C6,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B7&amp;" / "&amp;C7&amp;" = "&amp;IF(N(C7)=0,"-",TEXT(B7/C7,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B8&amp;" / "&amp;C8&amp;" = "&amp;IF(N(C8)=0,"-",TEXT(B8/C8,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B9&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B10&amp;"件"</f>
         <v>【1部12時半時報】9/28
 SL東京1部1課
 ■有効提案取得（自アポ）
 3 / 14 = 21.4%
 ■有効提案取得（IS）
 3 / 11 = 27.3%
+■有効提案取得（自アポ＋IS合算）
+6 / 25 = 24.0%
 ■当日提案取得数
 5件
 ■有効ヨミ取得数
@@ -2040,29 +2072,44 @@
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <f aca="false">入力!$I$9+入力!$I$10</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <f aca="false">入力!$I$7+入力!$I$8</f>
+        <v>25</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <f aca="false">IF(N(C8)=0,"-",B8/C8)</f>
+        <v>0.24</v>
+      </c>
+      <c r="F8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B9" s="16" t="n">
         <f aca="false">入力!$I$11</f>
         <v>5</v>
-      </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="F8" s="15"/>
-    </row>
-    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="16" t="n">
-        <f aca="false">入力!$I$12</f>
-        <v>3</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="F9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <f aca="false">入力!$I$12</f>
+        <v>3</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
       <c r="F10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2091,7 +2138,7 @@
         <v>【1部15時半時報】SL東京1部1課</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2108,13 +2155,15 @@
         <v>23</v>
       </c>
       <c r="F20" s="15" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"15時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B21&amp;" / "&amp;C21&amp;" = "&amp;IF(N(C21)=0,"-",TEXT(B21/C21,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B22&amp;" / "&amp;C22&amp;" = "&amp;IF(N(C22)=0,"-",TEXT(B22/C22,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B23&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B24&amp;"件"</f>
+        <f aca="false">"【"&amp;設定!$B$4&amp;"15時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B21&amp;" / "&amp;C21&amp;" = "&amp;IF(N(C21)=0,"-",TEXT(B21/C21,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B22&amp;" / "&amp;C22&amp;" = "&amp;IF(N(C22)=0,"-",TEXT(B22/C22,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B23&amp;" / "&amp;C23&amp;" = "&amp;IF(N(C23)=0,"-",TEXT(B23/C23,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B24&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B25&amp;"件"</f>
         <v>【1部15時半時報】9/28
 SL東京1部1課
 ■有効提案取得（自アポ）
 3 / 14 = 21.4%
 ■有効提案取得（IS）
 3 / 11 = 27.3%
+■有効提案取得（自アポ＋IS合算）
+6 / 25 = 24.0%
 ■当日提案取得数
 5件
 ■有効ヨミ取得数
@@ -2159,29 +2208,44 @@
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <f aca="false">入力!$I$9+入力!$I$17+入力!$I$10+入力!$I$18</f>
+        <v>6</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <f aca="false">入力!$I$7+入力!$I$15+入力!$I$8+入力!$I$16</f>
+        <v>25</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <f aca="false">IF(N(C23)=0,"-",B23/C23)</f>
+        <v>0.24</v>
+      </c>
+      <c r="F23" s="15"/>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B24" s="16" t="n">
         <f aca="false">入力!$I$11+入力!$I$19</f>
         <v>5</v>
-      </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="F23" s="15"/>
-    </row>
-    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" s="16" t="n">
-        <f aca="false">入力!$I$12+入力!$I$20</f>
-        <v>3</v>
       </c>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
       <c r="F24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="16" t="n">
+        <f aca="false">入力!$I$12+入力!$I$20</f>
+        <v>3</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
       <c r="F25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2231,31 +2295,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2263,7 +2327,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2271,7 +2335,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2279,7 +2343,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2287,7 +2351,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2295,7 +2359,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2312,7 +2376,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 提案訪問数 input, reduce to 12時/15時 reports, show 有効ヨミ rate in 課長報告
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2eWcGBYWFrU2WgTZUGmvP
</commit_message>
<xml_diff>
--- a/jiho/時報シート_SL東京1部1課.xlsx
+++ b/jiho/時報シート_SL東京1部1課.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="43">
   <si>
     <t xml:space="preserve">時報入力シート</t>
   </si>
@@ -33,15 +33,6 @@
     <t xml:space="preserve">【入力ルール】黄色セル＝手入力（その時間帯に発生した件数）／グレー＝自動計算。メンバー名は「設定」シートで変更します。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFC00000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">※ 〜</t>
-    </r>
     <r>
       <rPr>
         <sz val="9"/>
@@ -50,7 +41,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12:30</t>
+      <t xml:space="preserve">※ 12</t>
     </r>
     <r>
       <rPr>
@@ -59,7 +50,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">ブロックにはサンプル値が入っています。実運用時は上書き（または削除）してください。</t>
+      <t xml:space="preserve">時報告ブロックにはサンプル値が入っています。実運用時は上書き（または削除）してください。</t>
     </r>
   </si>
   <si>
@@ -71,7 +62,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【〜</t>
+      <t xml:space="preserve">【</t>
     </r>
     <r>
       <rPr>
@@ -82,7 +73,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12:30</t>
+      <t xml:space="preserve">12</t>
     </r>
     <r>
       <rPr>
@@ -92,94 +83,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">】</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">合計</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新規商談訪問数（自アポ）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">新規商談訪問数（</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IS</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">有効提案取得数（自アポ）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">有効提案取得数（</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IS</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">当日提案取得数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">有効ヨミ取得数</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【</t>
+      <t xml:space="preserve">時報告】（〜</t>
     </r>
     <r>
       <rPr>
@@ -190,7 +94,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12:30</t>
+      <t xml:space="preserve">12:00</t>
     </r>
     <r>
       <rPr>
@@ -200,7 +104,97 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">〜</t>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">合計</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新規商談訪問数（自アポ）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新規商談訪問数（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IS</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">有効提案取得数（自アポ）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得数（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IS</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">当日提案取得数</t>
+  </si>
+  <si>
+    <t xml:space="preserve">提案訪問数</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有効ヨミ取得数</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【</t>
     </r>
     <r>
       <rPr>
@@ -211,7 +205,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">15:30</t>
+      <t xml:space="preserve">15</t>
     </r>
     <r>
       <rPr>
@@ -221,19 +215,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">】</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【</t>
+      <t xml:space="preserve">時報告】（</t>
     </r>
     <r>
       <rPr>
@@ -244,7 +226,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">15:30</t>
+      <t xml:space="preserve">12:00</t>
     </r>
     <r>
       <rPr>
@@ -254,39 +236,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">〜終業】</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">【当日累計】（自動計算）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">有効提案取得率（自アポ）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">有効提案取得率（</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">IS</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
+      <t xml:space="preserve">15:00</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -294,14 +261,20 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">有効提案取得率（自アポ＋</t>
+    <t xml:space="preserve">【当日累計】（自動計算）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有効提案取得率（自アポ）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得率（</t>
     </r>
     <r>
       <rPr>
@@ -320,24 +293,18 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">合算）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課長報告シート（部長への時報）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">数値は「入力」シートから自動集計されます。右側の緑セルの文面をコピーして部長へ送信してください。</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">▼ 部長への報告文（</t>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得率（自アポ＋</t>
     </r>
     <r>
       <rPr>
@@ -347,42 +314,33 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時半）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">項目</t>
-  </si>
-  <si>
-    <t xml:space="preserve">件数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新規商談訪問数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">有効提案取得率</t>
-  </si>
-  <si>
-    <t xml:space="preserve">有効提案取得（自アポ）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">有効提案取得（</t>
+      <t xml:space="preserve">IS</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合算）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課長報告シート（部長への時報）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">数値は「入力」シートから自動集計されます。右側の緑セルの文面をコピーして部長へ送信してください。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">▼ 部長への報告文（</t>
     </r>
     <r>
       <rPr>
@@ -392,27 +350,42 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">IS</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">有効提案取得（自アポ＋</t>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">時）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">項目</t>
+  </si>
+  <si>
+    <t xml:space="preserve">件数</t>
+  </si>
+  <si>
+    <t xml:space="preserve">訪問数（分母）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">率</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有効提案取得（自アポ）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得（</t>
     </r>
     <r>
       <rPr>
@@ -431,18 +404,18 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">合算）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">▼ 部長への報告文（</t>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効提案取得（自アポ＋</t>
     </r>
     <r>
       <rPr>
@@ -452,6 +425,66 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">IS</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合算）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有効ヨミ取得数（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">÷</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">提案訪問数）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">▼ 部長への報告文（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">15</t>
     </r>
     <r>
@@ -461,7 +494,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">時半）</t>
+      <t xml:space="preserve">時）</t>
     </r>
   </si>
   <si>
@@ -677,15 +710,15 @@
     <font>
       <sz val="9"/>
       <color rgb="FFC00000"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFC00000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -1162,7 +1195,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -1368,82 +1401,92 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="10" t="n">
         <f aca="false">SUM(B12:H12)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="10" t="n">
+        <f aca="false">SUM(B13:H13)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="7" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="str">
         <f aca="false">IF(設定!B7="","",設定!B7)</f>
         <v>松下 魁翔</v>
       </c>
-      <c r="C14" s="7" t="str">
+      <c r="C15" s="7" t="str">
         <f aca="false">IF(設定!B8="","",設定!B8)</f>
         <v>中村 遼太</v>
       </c>
-      <c r="D14" s="7" t="str">
+      <c r="D15" s="7" t="str">
         <f aca="false">IF(設定!B9="","",設定!B9)</f>
         <v>加藤 真央</v>
       </c>
-      <c r="E14" s="7" t="str">
+      <c r="E15" s="7" t="str">
         <f aca="false">IF(設定!B10="","",設定!B10)</f>
         <v>大門 隼人</v>
       </c>
-      <c r="F14" s="7" t="str">
+      <c r="F15" s="7" t="str">
         <f aca="false">IF(設定!B11="","",設定!B11)</f>
         <v>杉本 賢亮</v>
       </c>
-      <c r="G14" s="7" t="str">
+      <c r="G15" s="7" t="str">
         <f aca="false">IF(設定!B12="","",設定!B12)</f>
         <v/>
       </c>
-      <c r="H14" s="7" t="str">
+      <c r="H15" s="7" t="str">
         <f aca="false">IF(設定!B13="","",設定!B13)</f>
         <v/>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I15" s="7" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="10" t="n">
-        <f aca="false">SUM(B15:H15)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -1459,7 +1502,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -1475,7 +1518,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -1491,7 +1534,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -1507,7 +1550,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1521,510 +1564,447 @@
         <v>0</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="10" t="n">
+        <f aca="false">SUM(B21:H21)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="7" t="str">
+      <c r="A22" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="10" t="n">
+        <f aca="false">SUM(B22:H22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" s="7" t="str">
         <f aca="false">IF(設定!B7="","",設定!B7)</f>
         <v>松下 魁翔</v>
       </c>
-      <c r="C22" s="7" t="str">
+      <c r="C24" s="7" t="str">
         <f aca="false">IF(設定!B8="","",設定!B8)</f>
         <v>中村 遼太</v>
       </c>
-      <c r="D22" s="7" t="str">
+      <c r="D24" s="7" t="str">
         <f aca="false">IF(設定!B9="","",設定!B9)</f>
         <v>加藤 真央</v>
       </c>
-      <c r="E22" s="7" t="str">
+      <c r="E24" s="7" t="str">
         <f aca="false">IF(設定!B10="","",設定!B10)</f>
         <v>大門 隼人</v>
       </c>
-      <c r="F22" s="7" t="str">
+      <c r="F24" s="7" t="str">
         <f aca="false">IF(設定!B11="","",設定!B11)</f>
         <v>杉本 賢亮</v>
       </c>
-      <c r="G22" s="7" t="str">
+      <c r="G24" s="7" t="str">
         <f aca="false">IF(設定!B12="","",設定!B12)</f>
         <v/>
       </c>
-      <c r="H22" s="7" t="str">
+      <c r="H24" s="7" t="str">
         <f aca="false">IF(設定!B13="","",設定!B13)</f>
         <v/>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I24" s="7" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="10" t="n">
-        <f aca="false">SUM(B23:H23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="10" t="n">
-        <f aca="false">SUM(B24:H24)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
+        <v>6</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <f aca="false">SUM(B7,B16)</f>
+        <v>3</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <f aca="false">SUM(C7,C16)</f>
+        <v>2</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <f aca="false">SUM(D7,D16)</f>
+        <v>4</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <f aca="false">SUM(E7,E16)</f>
+        <v>3</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <f aca="false">SUM(F7,F16)</f>
+        <v>2</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <f aca="false">SUM(G7,G16)</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="11" t="n">
+        <f aca="false">SUM(H7,H16)</f>
+        <v>0</v>
+      </c>
       <c r="I25" s="10" t="n">
         <f aca="false">SUM(B25:H25)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
+        <v>7</v>
+      </c>
+      <c r="B26" s="11" t="n">
+        <f aca="false">SUM(B8,B17)</f>
+        <v>2</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <f aca="false">SUM(C8,C17)</f>
+        <v>3</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <f aca="false">SUM(D8,D17)</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <f aca="false">SUM(E8,E17)</f>
+        <v>2</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <f aca="false">SUM(F8,F17)</f>
+        <v>3</v>
+      </c>
+      <c r="G26" s="11" t="n">
+        <f aca="false">SUM(G8,G17)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="11" t="n">
+        <f aca="false">SUM(H8,H17)</f>
+        <v>0</v>
+      </c>
       <c r="I26" s="10" t="n">
         <f aca="false">SUM(B26:H26)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
+        <v>8</v>
+      </c>
+      <c r="B27" s="11" t="n">
+        <f aca="false">SUM(B9,B18)</f>
+        <v>1</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <f aca="false">SUM(C9,C18)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <f aca="false">SUM(D9,D18)</f>
+        <v>1</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <f aca="false">SUM(E9,E18)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <f aca="false">SUM(F9,F18)</f>
+        <v>1</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <f aca="false">SUM(G9,G18)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="11" t="n">
+        <f aca="false">SUM(H9,H18)</f>
+        <v>0</v>
+      </c>
       <c r="I27" s="10" t="n">
         <f aca="false">SUM(B27:H27)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
+        <v>9</v>
+      </c>
+      <c r="B28" s="11" t="n">
+        <f aca="false">SUM(B10,B19)</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <f aca="false">SUM(C10,C19)</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <f aca="false">SUM(D10,D19)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <f aca="false">SUM(E10,E19)</f>
+        <v>1</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <f aca="false">SUM(F10,F19)</f>
+        <v>1</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <f aca="false">SUM(G10,G19)</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <f aca="false">SUM(H10,H19)</f>
+        <v>0</v>
+      </c>
       <c r="I28" s="10" t="n">
         <f aca="false">SUM(B28:H28)</f>
-        <v>0</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <f aca="false">SUM(B11,B20)</f>
+        <v>1</v>
+      </c>
+      <c r="C29" s="11" t="n">
+        <f aca="false">SUM(C11,C20)</f>
+        <v>1</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <f aca="false">SUM(D11,D20)</f>
+        <v>1</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <f aca="false">SUM(E11,E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <f aca="false">SUM(F11,F20)</f>
+        <v>2</v>
+      </c>
+      <c r="G29" s="11" t="n">
+        <f aca="false">SUM(G11,G20)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="11" t="n">
+        <f aca="false">SUM(H11,H20)</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <f aca="false">SUM(B29:H29)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" s="7" t="str">
-        <f aca="false">IF(設定!B7="","",設定!B7)</f>
-        <v>松下 魁翔</v>
-      </c>
-      <c r="C30" s="7" t="str">
-        <f aca="false">IF(設定!B8="","",設定!B8)</f>
-        <v>中村 遼太</v>
-      </c>
-      <c r="D30" s="7" t="str">
-        <f aca="false">IF(設定!B9="","",設定!B9)</f>
-        <v>加藤 真央</v>
-      </c>
-      <c r="E30" s="7" t="str">
-        <f aca="false">IF(設定!B10="","",設定!B10)</f>
-        <v>大門 隼人</v>
-      </c>
-      <c r="F30" s="7" t="str">
-        <f aca="false">IF(設定!B11="","",設定!B11)</f>
-        <v>杉本 賢亮</v>
-      </c>
-      <c r="G30" s="7" t="str">
-        <f aca="false">IF(設定!B12="","",設定!B12)</f>
-        <v/>
-      </c>
-      <c r="H30" s="7" t="str">
-        <f aca="false">IF(設定!B13="","",設定!B13)</f>
-        <v/>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>5</v>
+      <c r="A30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="11" t="n">
+        <f aca="false">SUM(B12,B21)</f>
+        <v>2</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <f aca="false">SUM(C12,C21)</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <f aca="false">SUM(D12,D21)</f>
+        <v>2</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <f aca="false">SUM(E12,E21)</f>
+        <v>1</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <f aca="false">SUM(F12,F21)</f>
+        <v>2</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <f aca="false">SUM(G12,G21)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <f aca="false">SUM(H12,H21)</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <f aca="false">SUM(B30:H30)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B31" s="11" t="n">
-        <f aca="false">SUM(B7,B15,B23)</f>
-        <v>3</v>
+        <f aca="false">SUM(B13,B22)</f>
+        <v>1</v>
       </c>
       <c r="C31" s="11" t="n">
-        <f aca="false">SUM(C7,C15,C23)</f>
-        <v>2</v>
+        <f aca="false">SUM(C13,C22)</f>
+        <v>0</v>
       </c>
       <c r="D31" s="11" t="n">
-        <f aca="false">SUM(D7,D15,D23)</f>
-        <v>4</v>
+        <f aca="false">SUM(D13,D22)</f>
+        <v>1</v>
       </c>
       <c r="E31" s="11" t="n">
-        <f aca="false">SUM(E7,E15,E23)</f>
-        <v>3</v>
+        <f aca="false">SUM(E13,E22)</f>
+        <v>1</v>
       </c>
       <c r="F31" s="11" t="n">
-        <f aca="false">SUM(F7,F15,F23)</f>
-        <v>2</v>
+        <f aca="false">SUM(F13,F22)</f>
+        <v>0</v>
       </c>
       <c r="G31" s="11" t="n">
-        <f aca="false">SUM(G7,G15,G23)</f>
+        <f aca="false">SUM(G13,G22)</f>
         <v>0</v>
       </c>
       <c r="H31" s="11" t="n">
-        <f aca="false">SUM(H7,H15,H23)</f>
+        <f aca="false">SUM(H13,H22)</f>
         <v>0</v>
       </c>
       <c r="I31" s="10" t="n">
         <f aca="false">SUM(B31:H31)</f>
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="11" t="n">
-        <f aca="false">SUM(B8,B16,B24)</f>
-        <v>2</v>
-      </c>
-      <c r="C32" s="11" t="n">
-        <f aca="false">SUM(C8,C16,C24)</f>
-        <v>3</v>
-      </c>
-      <c r="D32" s="11" t="n">
-        <f aca="false">SUM(D8,D16,D24)</f>
-        <v>1</v>
-      </c>
-      <c r="E32" s="11" t="n">
-        <f aca="false">SUM(E8,E16,E24)</f>
-        <v>2</v>
-      </c>
-      <c r="F32" s="11" t="n">
-        <f aca="false">SUM(F8,F16,F24)</f>
-        <v>3</v>
-      </c>
-      <c r="G32" s="11" t="n">
-        <f aca="false">SUM(G8,G16,G24)</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="11" t="n">
-        <f aca="false">SUM(H8,H16,H24)</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="10" t="n">
-        <f aca="false">SUM(B32:H32)</f>
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="B32" s="12" t="n">
+        <f aca="false">IF(N((B25))=0,"-",(B27)/(B25))</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <f aca="false">IF(N((C25))=0,"-",(C27)/(C25))</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="12" t="n">
+        <f aca="false">IF(N((D25))=0,"-",(D27)/(D25))</f>
+        <v>0.25</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <f aca="false">IF(N((E25))=0,"-",(E27)/(E25))</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <f aca="false">IF(N((F25))=0,"-",(F27)/(F25))</f>
+        <v>0.5</v>
+      </c>
+      <c r="G32" s="12" t="str">
+        <f aca="false">IF(N((G25))=0,"-",(G27)/(G25))</f>
+        <v>-</v>
+      </c>
+      <c r="H32" s="12" t="str">
+        <f aca="false">IF(N((H25))=0,"-",(H27)/(H25))</f>
+        <v>-</v>
+      </c>
+      <c r="I32" s="13" t="n">
+        <f aca="false">IF(N((I25))=0,"-",(I27)/(I25))</f>
+        <v>0.214285714285714</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="11" t="n">
-        <f aca="false">SUM(B9,B17,B25)</f>
-        <v>1</v>
-      </c>
-      <c r="C33" s="11" t="n">
-        <f aca="false">SUM(C9,C17,C25)</f>
-        <v>0</v>
-      </c>
-      <c r="D33" s="11" t="n">
-        <f aca="false">SUM(D9,D17,D25)</f>
-        <v>1</v>
-      </c>
-      <c r="E33" s="11" t="n">
-        <f aca="false">SUM(E9,E17,E25)</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="11" t="n">
-        <f aca="false">SUM(F9,F17,F25)</f>
-        <v>1</v>
-      </c>
-      <c r="G33" s="11" t="n">
-        <f aca="false">SUM(G9,G17,G25)</f>
-        <v>0</v>
-      </c>
-      <c r="H33" s="11" t="n">
-        <f aca="false">SUM(H9,H17,H25)</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="10" t="n">
-        <f aca="false">SUM(B33:H33)</f>
-        <v>3</v>
+        <v>16</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <f aca="false">IF(N((B26))=0,"-",(B28)/(B26))</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <f aca="false">IF(N((C26))=0,"-",(C28)/(C26))</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="D33" s="12" t="n">
+        <f aca="false">IF(N((D26))=0,"-",(D28)/(D26))</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">IF(N((E26))=0,"-",(E28)/(E26))</f>
+        <v>0.5</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <f aca="false">IF(N((F26))=0,"-",(F28)/(F26))</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G33" s="12" t="str">
+        <f aca="false">IF(N((G26))=0,"-",(G28)/(G26))</f>
+        <v>-</v>
+      </c>
+      <c r="H33" s="12" t="str">
+        <f aca="false">IF(N((H26))=0,"-",(H28)/(H26))</f>
+        <v>-</v>
+      </c>
+      <c r="I33" s="13" t="n">
+        <f aca="false">IF(N((I26))=0,"-",(I28)/(I26))</f>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B34" s="11" t="n">
-        <f aca="false">SUM(B10,B18,B26)</f>
-        <v>0</v>
-      </c>
-      <c r="C34" s="11" t="n">
-        <f aca="false">SUM(C10,C18,C26)</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="11" t="n">
-        <f aca="false">SUM(D10,D18,D26)</f>
-        <v>0</v>
-      </c>
-      <c r="E34" s="11" t="n">
-        <f aca="false">SUM(E10,E18,E26)</f>
-        <v>1</v>
-      </c>
-      <c r="F34" s="11" t="n">
-        <f aca="false">SUM(F10,F18,F26)</f>
-        <v>1</v>
-      </c>
-      <c r="G34" s="11" t="n">
-        <f aca="false">SUM(G10,G18,G26)</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="11" t="n">
-        <f aca="false">SUM(H10,H18,H26)</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="10" t="n">
-        <f aca="false">SUM(B34:H34)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="11" t="n">
-        <f aca="false">SUM(B11,B19,B27)</f>
-        <v>1</v>
-      </c>
-      <c r="C35" s="11" t="n">
-        <f aca="false">SUM(C11,C19,C27)</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="11" t="n">
-        <f aca="false">SUM(D11,D19,D27)</f>
-        <v>1</v>
-      </c>
-      <c r="E35" s="11" t="n">
-        <f aca="false">SUM(E11,E19,E27)</f>
-        <v>0</v>
-      </c>
-      <c r="F35" s="11" t="n">
-        <f aca="false">SUM(F11,F19,F27)</f>
-        <v>2</v>
-      </c>
-      <c r="G35" s="11" t="n">
-        <f aca="false">SUM(G11,G19,G27)</f>
-        <v>0</v>
-      </c>
-      <c r="H35" s="11" t="n">
-        <f aca="false">SUM(H11,H19,H27)</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="10" t="n">
-        <f aca="false">SUM(B35:H35)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" s="11" t="n">
-        <f aca="false">SUM(B12,B20,B28)</f>
-        <v>1</v>
-      </c>
-      <c r="C36" s="11" t="n">
-        <f aca="false">SUM(C12,C20,C28)</f>
-        <v>0</v>
-      </c>
-      <c r="D36" s="11" t="n">
-        <f aca="false">SUM(D12,D20,D28)</f>
-        <v>1</v>
-      </c>
-      <c r="E36" s="11" t="n">
-        <f aca="false">SUM(E12,E20,E28)</f>
-        <v>1</v>
-      </c>
-      <c r="F36" s="11" t="n">
-        <f aca="false">SUM(F12,F20,F28)</f>
-        <v>0</v>
-      </c>
-      <c r="G36" s="11" t="n">
-        <f aca="false">SUM(G12,G20,G28)</f>
-        <v>0</v>
-      </c>
-      <c r="H36" s="11" t="n">
-        <f aca="false">SUM(H12,H20,H28)</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="10" t="n">
-        <f aca="false">SUM(B36:H36)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B37" s="12" t="n">
-        <f aca="false">IF(N((B31))=0,"-",(B33)/(B31))</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="C37" s="12" t="n">
-        <f aca="false">IF(N((C31))=0,"-",(C33)/(C31))</f>
-        <v>0</v>
-      </c>
-      <c r="D37" s="12" t="n">
-        <f aca="false">IF(N((D31))=0,"-",(D33)/(D31))</f>
-        <v>0.25</v>
-      </c>
-      <c r="E37" s="12" t="n">
-        <f aca="false">IF(N((E31))=0,"-",(E33)/(E31))</f>
-        <v>0</v>
-      </c>
-      <c r="F37" s="12" t="n">
-        <f aca="false">IF(N((F31))=0,"-",(F33)/(F31))</f>
-        <v>0.5</v>
-      </c>
-      <c r="G37" s="12" t="str">
-        <f aca="false">IF(N((G31))=0,"-",(G33)/(G31))</f>
+        <v>17</v>
+      </c>
+      <c r="B34" s="12" t="n">
+        <f aca="false">IF(N((B25+B26))=0,"-",(B27+B28)/(B25+B26))</f>
+        <v>0.2</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <f aca="false">IF(N((C25+C26))=0,"-",(C27+C28)/(C25+C26))</f>
+        <v>0.2</v>
+      </c>
+      <c r="D34" s="12" t="n">
+        <f aca="false">IF(N((D25+D26))=0,"-",(D27+D28)/(D25+D26))</f>
+        <v>0.2</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <f aca="false">IF(N((E25+E26))=0,"-",(E27+E28)/(E25+E26))</f>
+        <v>0.2</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <f aca="false">IF(N((F25+F26))=0,"-",(F27+F28)/(F25+F26))</f>
+        <v>0.4</v>
+      </c>
+      <c r="G34" s="12" t="str">
+        <f aca="false">IF(N((G25+G26))=0,"-",(G27+G28)/(G25+G26))</f>
         <v>-</v>
       </c>
-      <c r="H37" s="12" t="str">
-        <f aca="false">IF(N((H31))=0,"-",(H33)/(H31))</f>
+      <c r="H34" s="12" t="str">
+        <f aca="false">IF(N((H25+H26))=0,"-",(H27+H28)/(H25+H26))</f>
         <v>-</v>
       </c>
-      <c r="I37" s="13" t="n">
-        <f aca="false">IF(N((I31))=0,"-",(I33)/(I31))</f>
-        <v>0.214285714285714</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B38" s="12" t="n">
-        <f aca="false">IF(N((B32))=0,"-",(B34)/(B32))</f>
-        <v>0</v>
-      </c>
-      <c r="C38" s="12" t="n">
-        <f aca="false">IF(N((C32))=0,"-",(C34)/(C32))</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="D38" s="12" t="n">
-        <f aca="false">IF(N((D32))=0,"-",(D34)/(D32))</f>
-        <v>0</v>
-      </c>
-      <c r="E38" s="12" t="n">
-        <f aca="false">IF(N((E32))=0,"-",(E34)/(E32))</f>
-        <v>0.5</v>
-      </c>
-      <c r="F38" s="12" t="n">
-        <f aca="false">IF(N((F32))=0,"-",(F34)/(F32))</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="G38" s="12" t="str">
-        <f aca="false">IF(N((G32))=0,"-",(G34)/(G32))</f>
-        <v>-</v>
-      </c>
-      <c r="H38" s="12" t="str">
-        <f aca="false">IF(N((H32))=0,"-",(H34)/(H32))</f>
-        <v>-</v>
-      </c>
-      <c r="I38" s="13" t="n">
-        <f aca="false">IF(N((I32))=0,"-",(I34)/(I32))</f>
-        <v>0.272727272727273</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B39" s="12" t="n">
-        <f aca="false">IF(N((B31+B32))=0,"-",(B33+B34)/(B31+B32))</f>
-        <v>0.2</v>
-      </c>
-      <c r="C39" s="12" t="n">
-        <f aca="false">IF(N((C31+C32))=0,"-",(C33+C34)/(C31+C32))</f>
-        <v>0.2</v>
-      </c>
-      <c r="D39" s="12" t="n">
-        <f aca="false">IF(N((D31+D32))=0,"-",(D33+D34)/(D31+D32))</f>
-        <v>0.2</v>
-      </c>
-      <c r="E39" s="12" t="n">
-        <f aca="false">IF(N((E31+E32))=0,"-",(E33+E34)/(E31+E32))</f>
-        <v>0.2</v>
-      </c>
-      <c r="F39" s="12" t="n">
-        <f aca="false">IF(N((F31+F32))=0,"-",(F33+F34)/(F31+F32))</f>
-        <v>0.4</v>
-      </c>
-      <c r="G39" s="12" t="str">
-        <f aca="false">IF(N((G31+G32))=0,"-",(G33+G34)/(G31+G32))</f>
-        <v>-</v>
-      </c>
-      <c r="H39" s="12" t="str">
-        <f aca="false">IF(N((H31+H32))=0,"-",(H33+H34)/(H31+H32))</f>
-        <v>-</v>
-      </c>
-      <c r="I39" s="13" t="n">
-        <f aca="false">IF(N((I31+I32))=0,"-",(I33+I34)/(I31+I32))</f>
+      <c r="I34" s="13" t="n">
+        <f aca="false">IF(N((I25+I26))=0,"-",(I27+I28)/(I25+I26))</f>
         <v>0.24</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" error="0以上の整数を入力してください" errorStyle="stop" errorTitle="入力エラー" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B7:H12 B15:H20 B23:H28" type="whole">
+    <dataValidation allowBlank="false" error="0以上の整数を入力してください" errorStyle="stop" errorTitle="入力エラー" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B7:H13 B16:H22" type="whole">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2065,8 +2045,8 @@
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"12時半時報】"&amp;設定!$B$3</f>
-        <v>【1部12時半時報】SL東京1部1課</v>
+        <f aca="false">"【"&amp;設定!$B$4&amp;"12時時報】"&amp;設定!$B$3</f>
+        <v>【1部12時時報】SL東京1部1課</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>20</v>
@@ -2086,8 +2066,8 @@
         <v>24</v>
       </c>
       <c r="F5" s="15" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"12時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B6&amp;" / "&amp;C6&amp;" = "&amp;IF(N(C6)=0,"-",TEXT(B6/C6,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B7&amp;" / "&amp;C7&amp;" = "&amp;IF(N(C7)=0,"-",TEXT(B7/C7,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B8&amp;" / "&amp;C8&amp;" = "&amp;IF(N(C8)=0,"-",TEXT(B8/C8,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B9&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B10&amp;"件"</f>
-        <v>【1部12時半時報】9/28
+        <f aca="false">"【"&amp;設定!$B$4&amp;"12時時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B6&amp;" / "&amp;C6&amp;" = "&amp;IF(N(C6)=0,"-",TEXT(B6/C6,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B7&amp;" / "&amp;C7&amp;" = "&amp;IF(N(C7)=0,"-",TEXT(B7/C7,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B8&amp;" / "&amp;C8&amp;" = "&amp;IF(N(C8)=0,"-",TEXT(B8/C8,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B9&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数（÷提案訪問数）"&amp;CHAR(10)&amp;B10&amp;" / "&amp;C10&amp;" = "&amp;IF(N(C10)=0,"-",TEXT(B10/C10,"0.0%"))</f>
+        <v>【1部12時時報】9/28
 SL東京1部1課
 ■有効提案取得（自アポ）
 3 / 14 = 21.4%
@@ -2097,8 +2077,8 @@
 6 / 25 = 24.0%
 ■当日提案取得数
 5件
-■有効ヨミ取得数
-3件</v>
+■有効ヨミ取得数（÷提案訪問数）
+3 / 8 = 37.5%</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2169,14 +2149,20 @@
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <f aca="false">入力!$I$13</f>
+        <v>3</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <f aca="false">入力!$I$12</f>
-        <v>3</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
+        <v>8</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <f aca="false">IF(N(C10)=0,"-",B10/C10)</f>
+        <v>0.375</v>
+      </c>
       <c r="F10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2201,11 +2187,11 @@
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"15時半時報】"&amp;設定!$B$3</f>
-        <v>【1部15時半時報】SL東京1部1課</v>
+        <f aca="false">"【"&amp;設定!$B$4&amp;"15時時報】"&amp;設定!$B$3</f>
+        <v>【1部15時時報】SL東京1部1課</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2222,8 +2208,8 @@
         <v>24</v>
       </c>
       <c r="F20" s="15" t="str">
-        <f aca="false">"【"&amp;設定!$B$4&amp;"15時半時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B21&amp;" / "&amp;C21&amp;" = "&amp;IF(N(C21)=0,"-",TEXT(B21/C21,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B22&amp;" / "&amp;C22&amp;" = "&amp;IF(N(C22)=0,"-",TEXT(B22/C22,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B23&amp;" / "&amp;C23&amp;" = "&amp;IF(N(C23)=0,"-",TEXT(B23/C23,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B24&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数"&amp;CHAR(10)&amp;B25&amp;"件"</f>
-        <v>【1部15時半時報】9/28
+        <f aca="false">"【"&amp;設定!$B$4&amp;"15時時報】"&amp;TEXT(入力!$B$2,"m/d")&amp;CHAR(10)&amp;設定!$B$3&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ）"&amp;CHAR(10)&amp;B21&amp;" / "&amp;C21&amp;" = "&amp;IF(N(C21)=0,"-",TEXT(B21/C21,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（IS）"&amp;CHAR(10)&amp;B22&amp;" / "&amp;C22&amp;" = "&amp;IF(N(C22)=0,"-",TEXT(B22/C22,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効提案取得（自アポ＋IS合算）"&amp;CHAR(10)&amp;B23&amp;" / "&amp;C23&amp;" = "&amp;IF(N(C23)=0,"-",TEXT(B23/C23,"0.0%"))&amp;CHAR(10)&amp;CHAR(10)&amp;"■当日提案取得数"&amp;CHAR(10)&amp;B24&amp;"件"&amp;CHAR(10)&amp;CHAR(10)&amp;"■有効ヨミ取得数（÷提案訪問数）"&amp;CHAR(10)&amp;B25&amp;" / "&amp;C25&amp;" = "&amp;IF(N(C25)=0,"-",TEXT(B25/C25,"0.0%"))</f>
+        <v>【1部15時時報】9/28
 SL東京1部1課
 ■有効提案取得（自アポ）
 3 / 14 = 21.4%
@@ -2233,8 +2219,8 @@
 6 / 25 = 24.0%
 ■当日提案取得数
 5件
-■有効ヨミ取得数
-3件</v>
+■有効ヨミ取得数（÷提案訪問数）
+3 / 8 = 37.5%</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2242,11 +2228,11 @@
         <v>25</v>
       </c>
       <c r="B21" s="11" t="n">
-        <f aca="false">入力!$I$9+入力!$I$17</f>
+        <f aca="false">入力!$I$9+入力!$I$18</f>
         <v>3</v>
       </c>
       <c r="C21" s="11" t="n">
-        <f aca="false">入力!$I$7+入力!$I$15</f>
+        <f aca="false">入力!$I$7+入力!$I$16</f>
         <v>14</v>
       </c>
       <c r="D21" s="12" t="n">
@@ -2260,11 +2246,11 @@
         <v>26</v>
       </c>
       <c r="B22" s="11" t="n">
-        <f aca="false">入力!$I$10+入力!$I$18</f>
+        <f aca="false">入力!$I$10+入力!$I$19</f>
         <v>3</v>
       </c>
       <c r="C22" s="11" t="n">
-        <f aca="false">入力!$I$8+入力!$I$16</f>
+        <f aca="false">入力!$I$8+入力!$I$17</f>
         <v>11</v>
       </c>
       <c r="D22" s="12" t="n">
@@ -2278,11 +2264,11 @@
         <v>27</v>
       </c>
       <c r="B23" s="11" t="n">
-        <f aca="false">入力!$I$9+入力!$I$17+入力!$I$10+入力!$I$18</f>
+        <f aca="false">入力!$I$9+入力!$I$18+入力!$I$10+入力!$I$19</f>
         <v>6</v>
       </c>
       <c r="C23" s="11" t="n">
-        <f aca="false">入力!$I$7+入力!$I$15+入力!$I$8+入力!$I$16</f>
+        <f aca="false">入力!$I$7+入力!$I$16+入力!$I$8+入力!$I$17</f>
         <v>25</v>
       </c>
       <c r="D23" s="12" t="n">
@@ -2296,7 +2282,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="16" t="n">
-        <f aca="false">入力!$I$11+入力!$I$19</f>
+        <f aca="false">入力!$I$11+入力!$I$20</f>
         <v>5</v>
       </c>
       <c r="C24" s="11"/>
@@ -2305,14 +2291,20 @@
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" s="16" t="n">
-        <f aca="false">入力!$I$12+入力!$I$20</f>
+        <v>28</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <f aca="false">入力!$I$13+入力!$I$22</f>
         <v>3</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
+      <c r="C25" s="11" t="n">
+        <f aca="false">入力!$I$12+入力!$I$21</f>
+        <v>8</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <f aca="false">IF(N(C25)=0,"-",B25/C25)</f>
+        <v>0.375</v>
+      </c>
       <c r="F25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2362,31 +2354,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2394,7 +2386,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2402,7 +2394,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,7 +2402,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2418,7 +2410,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2426,7 +2418,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2443,7 +2435,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>